<commit_message>
Set CII membership cost to N/A.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -4204,7 +4204,7 @@
         </is>
       </c>
       <c r="B35" s="64" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="C35" s="50" t="inlineStr">
         <is>
@@ -4213,12 +4213,12 @@
       </c>
       <c r="D35" s="50" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E35" s="56" t="inlineStr">
         <is>
-          <t>Cert CII (MP) ongoing.</t>
+          <t>Not applicable — set to £0 by Robert.</t>
         </is>
       </c>
       <c r="F35" s="66">

</xml_diff>

<commit_message>
Recast 2027 targets to 40 leads, 30 spoken, 1-in-3 conversion.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -447,7 +447,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -678,6 +678,13 @@
     <xf numFmtId="164" fontId="9" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2009,12 +2016,36 @@
       </c>
     </row>
     <row r="39" ht="36" customHeight="1">
-      <c r="A39" s="86" t="n"/>
-      <c r="B39" s="86" t="n"/>
-      <c r="C39" s="86" t="n"/>
-      <c r="D39" s="86" t="n"/>
-      <c r="E39" s="90" t="n"/>
-      <c r="F39" s="86" t="n"/>
+      <c r="A39" s="49" t="inlineStr">
+        <is>
+          <t>Planning conversion model</t>
+        </is>
+      </c>
+      <c r="B39" s="49" t="inlineStr">
+        <is>
+          <t>40 leads → 30 spoken</t>
+        </is>
+      </c>
+      <c r="C39" s="49" t="inlineStr">
+        <is>
+          <t>All sources combined</t>
+        </is>
+      </c>
+      <c r="D39" s="49" t="inlineStr">
+        <is>
+          <t>40 leads a month</t>
+        </is>
+      </c>
+      <c r="E39" s="89" t="inlineStr">
+        <is>
+          <t>1 in 3 of 30 spoken (10 completions)</t>
+        </is>
+      </c>
+      <c r="F39" s="49" t="inlineStr">
+        <is>
+          <t>Drives Financial Plan written target</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="36" customHeight="1">
       <c r="A40" s="86" t="n"/>
@@ -2747,7 +2778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P24"/>
+  <dimension ref="A1:P35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2808,15 +2839,16 @@
           <t>Mortgage</t>
         </is>
       </c>
-      <c r="B7" s="91" t="n">
-        <v>790000</v>
+      <c r="B7" s="92">
+        <f>B33</f>
+        <v/>
       </c>
       <c r="C7" s="36" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="38" t="inlineStr">
         <is>
-          <t>Named sources only (DJ Alexander + Thorntons). Mid-point of 3–5 completions × £180k–£250k. Income = 0.35% of this written amount.</t>
+          <t>40 leads → 30 spoken → 1 in 3 = 10 completions × £180k–£250k (mid £215k). Income = 0.35% of written. Change yellow cells in the conversion model below.</t>
         </is>
       </c>
       <c r="E7" s="40" t="n"/>
@@ -2828,15 +2860,16 @@
           <t>Protection</t>
         </is>
       </c>
-      <c r="B8" s="91" t="n">
-        <v>2000</v>
+      <c r="B8" s="92">
+        <f>B35</f>
+        <v/>
       </c>
       <c r="C8" s="36" t="n">
         <v>2</v>
       </c>
       <c r="D8" s="38" t="inlineStr">
         <is>
-          <t>Cash: £1,000 per protection case; 1–3 cases a month (mid £2,000). Not a large written-volume figure.</t>
+          <t>£1,000 per protection case; 1 in 3 of the 10 completions ≈ 3 cases. Linked to the conversion model.</t>
         </is>
       </c>
       <c r="E8" s="40" t="n"/>
@@ -3367,16 +3400,206 @@
         <v/>
       </c>
     </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="93" t="inlineStr">
+        <is>
+          <t>Conversion model (plan target)</t>
+        </is>
+      </c>
+      <c r="B26" s="61" t="n"/>
+      <c r="C26" s="61" t="n"/>
+      <c r="D26" s="61" t="n"/>
+      <c r="E26" s="61" t="n"/>
+      <c r="F26" s="61" t="n"/>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="72" t="inlineStr">
+        <is>
+          <t>Driver</t>
+        </is>
+      </c>
+      <c r="B27" s="72" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C27" s="72" t="inlineStr">
+        <is>
+          <t>Unit / note</t>
+        </is>
+      </c>
+      <c r="D27" s="94" t="n"/>
+      <c r="E27" s="94" t="n"/>
+      <c r="F27" s="94" t="n"/>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="63" t="inlineStr">
+        <is>
+          <t>Leads in a month</t>
+        </is>
+      </c>
+      <c r="B28" s="49" t="n">
+        <v>40</v>
+      </c>
+      <c r="C28" s="87" t="inlineStr">
+        <is>
+          <t>Inbound leads</t>
+        </is>
+      </c>
+      <c r="D28" s="76" t="n"/>
+      <c r="E28" s="76" t="n"/>
+      <c r="F28" s="76" t="n"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="63" t="inlineStr">
+        <is>
+          <t>Spoken with</t>
+        </is>
+      </c>
+      <c r="B29" s="49" t="n">
+        <v>30</v>
+      </c>
+      <c r="C29" s="87" t="inlineStr">
+        <is>
+          <t>Appointments / conversations from those leads</t>
+        </is>
+      </c>
+      <c r="D29" s="76" t="n"/>
+      <c r="E29" s="76" t="n"/>
+      <c r="F29" s="76" t="n"/>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="63" t="inlineStr">
+        <is>
+          <t>Conversion of spoken (1 in n)</t>
+        </is>
+      </c>
+      <c r="B30" s="49" t="n">
+        <v>3</v>
+      </c>
+      <c r="C30" s="87" t="inlineStr">
+        <is>
+          <t>1 in 3 of the 30 spoken</t>
+        </is>
+      </c>
+      <c r="D30" s="76" t="n"/>
+      <c r="E30" s="76" t="n"/>
+      <c r="F30" s="76" t="n"/>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="63" t="inlineStr">
+        <is>
+          <t>Completions</t>
+        </is>
+      </c>
+      <c r="B31" s="67">
+        <f>B29/B30</f>
+        <v/>
+      </c>
+      <c r="C31" s="87" t="inlineStr">
+        <is>
+          <t>Spoken ÷ conversion = 10 cases</t>
+        </is>
+      </c>
+      <c r="D31" s="76" t="n"/>
+      <c r="E31" s="76" t="n"/>
+      <c r="F31" s="76" t="n"/>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="63" t="inlineStr">
+        <is>
+          <t>Average loan (mid of £180k–£250k)</t>
+        </is>
+      </c>
+      <c r="B32" s="55" t="n">
+        <v>215000</v>
+      </c>
+      <c r="C32" s="87" t="inlineStr">
+        <is>
+          <t>Overwrite if you want low £180k or high £250k</t>
+        </is>
+      </c>
+      <c r="D32" s="76" t="n"/>
+      <c r="E32" s="76" t="n"/>
+      <c r="F32" s="76" t="n"/>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="63" t="inlineStr">
+        <is>
+          <t>Mortgage written (feeds B7)</t>
+        </is>
+      </c>
+      <c r="B33" s="75">
+        <f>B31*B32</f>
+        <v/>
+      </c>
+      <c r="C33" s="87" t="inlineStr">
+        <is>
+          <t>10 × average loan</t>
+        </is>
+      </c>
+      <c r="D33" s="76" t="n"/>
+      <c r="E33" s="76" t="n"/>
+      <c r="F33" s="76" t="n"/>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="63" t="inlineStr">
+        <is>
+          <t>Mortgage income at 0.35% (before network)</t>
+        </is>
+      </c>
+      <c r="B34" s="75">
+        <f>B33*0.0035</f>
+        <v/>
+      </c>
+      <c r="C34" s="87" t="inlineStr">
+        <is>
+          <t>Not banked cash until the 2-month lag</t>
+        </is>
+      </c>
+      <c r="D34" s="76" t="n"/>
+      <c r="E34" s="76" t="n"/>
+      <c r="F34" s="76" t="n"/>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="63" t="inlineStr">
+        <is>
+          <t>Protection cases (1 in 3 completions × £1,000)</t>
+        </is>
+      </c>
+      <c r="B35" s="75">
+        <f>ROUND(B31/3,0)*1000</f>
+        <v/>
+      </c>
+      <c r="C35" s="87" t="inlineStr">
+        <is>
+          <t>About 3 cases → £3,000 (feeds B8)</t>
+        </is>
+      </c>
+      <c r="D35" s="76" t="n"/>
+      <c r="E35" s="76" t="n"/>
+      <c r="F35" s="76" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="19">
+    <mergeCell ref="A1:P2"/>
+    <mergeCell ref="C32:F32"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="D7:F7"/>
+    <mergeCell ref="C28:F28"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="C30:F30"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="C33:F33"/>
+    <mergeCell ref="D8:F8"/>
     <mergeCell ref="A11:P11"/>
     <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A1:P2"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="C35:F35"/>
+    <mergeCell ref="C29:F29"/>
+    <mergeCell ref="C31:F31"/>
     <mergeCell ref="A3:P3"/>
-    <mergeCell ref="D7:F7"/>
-    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="C27:F27"/>
     <mergeCell ref="D6:F6"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
@@ -3622,17 +3845,18 @@
           <t>Protection cash commission (monthly, before retention)</t>
         </is>
       </c>
-      <c r="B13" s="70" t="n">
-        <v>2000</v>
+      <c r="B13" s="70">
+        <f>'Financial Plan'!B8</f>
+        <v/>
       </c>
       <c r="C13" s="50" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Linked</t>
         </is>
       </c>
       <c r="D13" s="56" t="inlineStr">
         <is>
-          <t>Robert: £1,000 per case, 1–3 cases a month. Mid-point £2,000 cash before 15% retention.</t>
+          <t>£1,000 × ~3 protection cases from 10 completions (1 in 3). Linked to conversion model.</t>
         </is>
       </c>
       <c r="E13" s="56" t="inlineStr">
@@ -5750,7 +5974,7 @@
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="49" t="inlineStr">
         <is>
-          <t>Deliver £12.42m mortgage and £2.88m protection written (Financial Plan targets)</t>
+          <t>Deliver conversion model: 40 leads → 30 spoken → 10 completions; mortgage written from Financial Plan</t>
         </is>
       </c>
       <c r="B7" s="77" t="n"/>
@@ -5788,7 +6012,7 @@
     <row r="9" ht="36" customHeight="1">
       <c r="A9" s="49" t="inlineStr">
         <is>
-          <t>Convert DJ Alexander, Hannah Fraser and Ralph’s Thayer into live introducer flow</t>
+          <t>Run DJ Alexander and Thorntons as live introducers; system source TBC toward the 40-lead month</t>
         </is>
       </c>
       <c r="B9" s="77" t="n"/>
@@ -6186,7 +6410,7 @@
       </c>
       <c r="C6" s="49" t="inlineStr">
         <is>
-          <t>Launch Duncan &amp; Co; hit written targets and build toward £80–120k net cash.</t>
+          <t>Launch Duncan &amp; Co; hit the 40 / 30 / 1-in-3 conversion model (10 completions; written from Financial Plan) and build year-1 cash.</t>
         </is>
       </c>
       <c r="D6" s="49" t="inlineStr">
@@ -6322,7 +6546,7 @@
       </c>
       <c r="B9" s="49" t="inlineStr">
         <is>
-          <t>Rosemount protection workshops fortnightly; 15% net retention. Written target £240k/month is NOT cash.</t>
+          <t>Protection at £1,000 a case; 1 in 3 of mortgage completions. Network 15% retention.</t>
         </is>
       </c>
       <c r="C9" s="49" t="inlineStr">
@@ -6369,7 +6593,7 @@
       </c>
       <c r="B10" s="49" t="inlineStr">
         <is>
-          <t>No GI book. Other Income starter £1,500/month covers GI, referrals and Beanstalk JISA.</t>
+          <t>No GI book. Other Income set to £0 for 2027 until a route is agreed.</t>
         </is>
       </c>
       <c r="C10" s="49" t="inlineStr">
@@ -6609,7 +6833,7 @@
       </c>
       <c r="C15" s="49" t="inlineStr">
         <is>
-          <t>£18k Other Income across GI, Beanstalk, accountant intros and agreed referrals.</t>
+          <t>Other Income held at £0 unless a GI / referral route is switched on.</t>
         </is>
       </c>
       <c r="D15" s="49" t="inlineStr">

</xml_diff>